<commit_message>
Ariba webform filled as expected by UvA inkoop, including `Supplier part number`, prices before VAT, and Name including part number and beginning of description. Chrome.bat opens UvA's inkoop page. Specified old WBS, so nobody can order by chance on our grants.
</commit_message>
<xml_diff>
--- a/PaymentAndShipping.xlsx
+++ b/PaymentAndShipping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Florian\Labor\orders\QuickAriba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2609E7D0-ED46-4D05-968E-F8536C28F8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A249798-4C61-4A7A-8C3B-D94AC9F7AA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4296" yWindow="2754" windowWidth="17100" windowHeight="9900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23790" yWindow="-13590" windowWidth="17280" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -31,13 +31,13 @@
     <t>WBS</t>
   </si>
   <si>
-    <t>C.2329.0334</t>
-  </si>
-  <si>
     <t>SP D0.134</t>
   </si>
   <si>
     <t>20.4.2026</t>
+  </si>
+  <si>
+    <t>C.2329.0407</t>
   </si>
 </sst>
 </file>
@@ -396,13 +396,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added "deliver.bat" that only fills out the missing data on the delivery page. This is useful to place catalog orders.
</commit_message>
<xml_diff>
--- a/PaymentAndShipping.xlsx
+++ b/PaymentAndShipping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Florian\Labor\orders\QuickAriba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A249798-4C61-4A7A-8C3B-D94AC9F7AA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA775CD-A097-49E7-AF13-8304B685412D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23790" yWindow="-13590" windowWidth="17280" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="12683" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -31,13 +31,13 @@
     <t>WBS</t>
   </si>
   <si>
-    <t>SP D0.134</t>
-  </si>
-  <si>
-    <t>20.4.2026</t>
-  </si>
-  <si>
-    <t>C.2329.0407</t>
+    <t>C.2329.0425</t>
+  </si>
+  <si>
+    <t>SP D0.138</t>
+  </si>
+  <si>
+    <t>17.8.2026</t>
   </si>
 </sst>
 </file>
@@ -378,12 +378,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="3" width="21.89453125" customWidth="1"/>
+    <col min="1" max="3" width="21.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -394,15 +394,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>